<commit_message>
Translation keys added for manage obligations page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/december-waste/xlsx/02-select-single-prn.xlsx
+++ b/translations/welsh-translations/december-waste/xlsx/02-select-single-prn.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -147,92 +147,134 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="51" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx::accepted_towards_recycling_obligations</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accepted_towards_recycling_obligations</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-select-single</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/selected-prn/{id}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted towards {0} recycling obligations</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=2012-26252</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="51" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx::acceptance_year</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t xml:space="preserve">acceptance_year</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t xml:space="preserve">prns-select-single</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t xml:space="preserve">/report-data/selected-prn/{id}</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t xml:space="preserve">Can be accepted towards {0}</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=2012-26252</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="51" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx::acceptance_years</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">acceptance_years</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-select-single</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/selected-prn/{id}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Can be accepted towards {0} or {1}</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx::acceptance_years</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectSinglePrn.en.resx</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">acceptance_years</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">prns-select-single</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">/report-data/selected-prn/{id}</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Can be accepted towards {0} or {1}</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=2012-26252</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H7"/>
+  <autoFilter ref="A5:H8"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>